<commit_message>
Making plots for my personal data and writing captions.
</commit_message>
<xml_diff>
--- a/data/Data_Project_Water_Idea_HW3.xlsx
+++ b/data/Data_Project_Water_Idea_HW3.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/danielmatthys/github/ENVS-193DS_homework-03/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{971BA5D8-F40C-0A4E-AE82-46A6BDDF0AA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E7DCB68-36FA-494C-A1E9-C09F35E555E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2080" yWindow="520" windowWidth="28800" windowHeight="16100" xr2:uid="{FA6642B7-84E0-0D4F-B218-18AD033CFE33}"/>
+    <workbookView xWindow="4240" yWindow="3540" windowWidth="28800" windowHeight="16100" xr2:uid="{FA6642B7-84E0-0D4F-B218-18AD033CFE33}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet2" sheetId="2" r:id="rId1"/>

</xml_diff>

<commit_message>
Added captions for my visualizations, description for my affective visualization, and responded to parts of problem 4
</commit_message>
<xml_diff>
--- a/data/Data_Project_Water_Idea_HW3.xlsx
+++ b/data/Data_Project_Water_Idea_HW3.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/danielmatthys/github/ENVS-193DS_homework-03/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E7DCB68-36FA-494C-A1E9-C09F35E555E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F8A436A-1B3D-7342-B093-911129FCF180}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4240" yWindow="3540" windowWidth="28800" windowHeight="16100" xr2:uid="{FA6642B7-84E0-0D4F-B218-18AD033CFE33}"/>
+    <workbookView xWindow="7120" yWindow="580" windowWidth="28800" windowHeight="16100" xr2:uid="{FA6642B7-84E0-0D4F-B218-18AD033CFE33}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet2" sheetId="2" r:id="rId1"/>

</xml_diff>

<commit_message>
Loading in personal data
</commit_message>
<xml_diff>
--- a/data/Data_Project_Water_Idea_HW3.xlsx
+++ b/data/Data_Project_Water_Idea_HW3.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/danielmatthys/github/ENVS-193DS_homework-03/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F8A436A-1B3D-7342-B093-911129FCF180}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB35B320-6CFD-6C4A-A062-C31C5B9D3061}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7120" yWindow="580" windowWidth="28800" windowHeight="16100" xr2:uid="{FA6642B7-84E0-0D4F-B218-18AD033CFE33}"/>
+    <workbookView xWindow="0" yWindow="540" windowWidth="28800" windowHeight="16100" xr2:uid="{FA6642B7-84E0-0D4F-B218-18AD033CFE33}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet2" sheetId="2" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="47">
   <si>
     <t>Date</t>
   </si>
@@ -175,6 +175,9 @@
   </si>
   <si>
     <t>3.50</t>
+  </si>
+  <si>
+    <t>3.09</t>
   </si>
 </sst>
 </file>
@@ -1200,8 +1203,27 @@
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="C29" s="1"/>
-      <c r="G29" s="2"/>
+      <c r="A29" s="3">
+        <v>46084</v>
+      </c>
+      <c r="B29">
+        <v>64</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="D29" s="4">
+        <v>0.38541666666666669</v>
+      </c>
+      <c r="E29" t="s">
+        <v>16</v>
+      </c>
+      <c r="F29">
+        <v>2</v>
+      </c>
+      <c r="G29" s="2" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.2">
       <c r="C30" s="1"/>

</xml_diff>

<commit_message>
Committing all of my code and data
</commit_message>
<xml_diff>
--- a/data/Data_Project_Water_Idea_HW3.xlsx
+++ b/data/Data_Project_Water_Idea_HW3.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/danielmatthys/github/ENVS-193DS_homework-03/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB35B320-6CFD-6C4A-A062-C31C5B9D3061}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A78E2A3-4E77-B143-81CA-9CF3C2C707D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="540" windowWidth="28800" windowHeight="16100" xr2:uid="{FA6642B7-84E0-0D4F-B218-18AD033CFE33}"/>
+    <workbookView xWindow="9740" yWindow="560" windowWidth="28800" windowHeight="16100" xr2:uid="{FA6642B7-84E0-0D4F-B218-18AD033CFE33}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet2" sheetId="2" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="47">
   <si>
     <t>Date</t>
   </si>
@@ -1226,8 +1226,27 @@
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="C30" s="1"/>
-      <c r="G30" s="2"/>
+      <c r="A30" s="3">
+        <v>46085</v>
+      </c>
+      <c r="B30">
+        <v>61</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D30" s="4">
+        <v>0.34375</v>
+      </c>
+      <c r="E30" t="s">
+        <v>16</v>
+      </c>
+      <c r="F30">
+        <v>2</v>
+      </c>
+      <c r="G30" s="2" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.2">
       <c r="C31" s="1"/>

</xml_diff>